<commit_message>
Make Aeroflot weekly mood comments rotate and feel more personal
Expand lavender-raf narrative pools, seed variants by week end date,
and weave in week-specific stats (top line, late averages, payment peaks).
Also refresh cover epigraph and summary subtitle each week.

Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Аэрофлот статус 07.08.2026.xlsx
+++ b/output/Аэрофлот статус 07.08.2026.xlsx
@@ -1410,7 +1410,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>мягкий лавандовый раф: эспрессо, сливки и цветочный аромат — тот же уют, только в отчёте по заказам ♡</t>
+          <t>этот отчёт пахнет перроном на закате и свежей пенкой. Аэрофлот, мы рядом — даже когда сроки гуляют ✈️♡</t>
         </is>
       </c>
       <c r="K30" s="5" t="n"/>
@@ -1772,7 +1772,7 @@
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
@@ -1789,7 +1789,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Период: 31.07.2026 — 07.08.2026</t>
+          <t>Период: 31.07.2026 — 07.08.2026  ·  курс лавандовый, турбулентность эмоциональная — низкая</t>
         </is>
       </c>
     </row>
@@ -1801,14 +1801,14 @@
       </c>
       <c r="O4" s="24" t="inlineStr">
         <is>
-          <t>🌷 Спокойная, но уверенная неделя</t>
+          <t>🌤️ Мягкая ясная неделя</t>
         </is>
       </c>
       <c r="P4" s="25" t="n"/>
       <c r="Q4" s="25" t="n"/>
       <c r="R4" s="25" t="n"/>
     </row>
-    <row r="5" ht="18" customHeight="1">
+    <row r="5" ht="20" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Количество: 11   |   Сумма: 72,188.00 USD</t>
@@ -1816,14 +1816,14 @@
       </c>
       <c r="O5" s="27" t="inlineStr">
         <is>
-          <t>11 новых позиций на 72,188 USD. Без лишнего шума, зато с ароматом лаванды и пользой для клиента 💜</t>
+          <t>11 заказов, 72 188 USD. Ни бури, ни скуки — именно такой прогноз любит нежный отчёт 💜🌸</t>
         </is>
       </c>
       <c r="P5" s="28" t="n"/>
       <c r="Q5" s="28" t="n"/>
       <c r="R5" s="28" t="n"/>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>№ счета</t>
@@ -1874,7 +1874,7 @@
       <c r="Q6" s="28" t="n"/>
       <c r="R6" s="28" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7" ht="20" customHeight="1">
       <c r="A7" s="29" t="inlineStr">
         <is>
           <t>7082615150-4</t>
@@ -1917,7 +1917,7 @@
       <c r="Q7" s="28" t="n"/>
       <c r="R7" s="28" t="n"/>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="29" t="n">
         <v>7082613274</v>
       </c>
@@ -1958,7 +1958,7 @@
       <c r="Q8" s="28" t="n"/>
       <c r="R8" s="28" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" s="29" t="n">
         <v>6082615184</v>
       </c>
@@ -1995,6 +1995,10 @@
           <t>P20437126</t>
         </is>
       </c>
+      <c r="O9" s="28" t="n"/>
+      <c r="P9" s="28" t="n"/>
+      <c r="Q9" s="28" t="n"/>
+      <c r="R9" s="28" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="29" t="n">
@@ -2312,14 +2316,14 @@
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>🌙 Главное — доехали</t>
+          <t>🌙 Главное — долетели</t>
         </is>
       </c>
       <c r="P20" s="25" t="n"/>
       <c r="Q20" s="25" t="n"/>
       <c r="R20" s="25" t="n"/>
     </row>
-    <row r="21" ht="18" customHeight="1">
+    <row r="21" ht="20" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Количество: 35   |   Сумма: 283,812.20 USD</t>
@@ -2327,14 +2331,14 @@
       </c>
       <c r="O21" s="27" t="inlineStr">
         <is>
-          <t>Из 35 отгрузок много с опозданием (34). Ничего страшного: лаванда не торопится, а мы бережно доводим поставки. Клиент всё равно получит заботу 🫶</t>
+          <t>Из 35 отгрузок (283 812 USD) с опозданием 34, в среднем на ~21 дн., рекорд 68 дн.. Дышим глубже: детали всё равно нашли путь к клиенту. Лаванда не торопит — она сопровождает 🫶💜</t>
         </is>
       </c>
       <c r="P21" s="28" t="n"/>
       <c r="Q21" s="28" t="n"/>
       <c r="R21" s="28" t="n"/>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22" ht="20" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>№ счета</t>
@@ -2405,7 +2409,7 @@
       <c r="Q22" s="28" t="n"/>
       <c r="R22" s="28" t="n"/>
     </row>
-    <row r="23" ht="18" customHeight="1">
+    <row r="23" ht="20" customHeight="1">
       <c r="A23" s="29" t="inlineStr">
         <is>
           <t>250615100-4</t>
@@ -2464,7 +2468,7 @@
       <c r="Q23" s="28" t="n"/>
       <c r="R23" s="28" t="n"/>
     </row>
-    <row r="24" ht="18" customHeight="1">
+    <row r="24" ht="20" customHeight="1">
       <c r="A24" s="29" t="inlineStr">
         <is>
           <t>2072615550-4</t>
@@ -2523,7 +2527,7 @@
       <c r="Q24" s="28" t="n"/>
       <c r="R24" s="28" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="29" t="inlineStr">
         <is>
           <t>2072615550-4</t>
@@ -2577,6 +2581,10 @@
           <t>дата поставки в периоде; дата из BC</t>
         </is>
       </c>
+      <c r="O25" s="28" t="n"/>
+      <c r="P25" s="28" t="n"/>
+      <c r="Q25" s="28" t="n"/>
+      <c r="R25" s="28" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
@@ -4341,14 +4349,14 @@
       </c>
       <c r="O60" s="24" t="inlineStr">
         <is>
-          <t>🥛 Деньги капают — и это мило</t>
+          <t>🍯 Ложечка сливок в кассу</t>
         </is>
       </c>
       <c r="P60" s="25" t="n"/>
       <c r="Q60" s="25" t="n"/>
       <c r="R60" s="25" t="n"/>
     </row>
-    <row r="61" ht="18" customHeight="1">
+    <row r="61" ht="20" customHeight="1">
       <c r="A61" s="26" t="inlineStr">
         <is>
           <t>Количество: 6   |   Оплачено за период: 80,450.00 USD</t>
@@ -4356,14 +4364,14 @@
       </c>
       <c r="O61" s="27" t="inlineStr">
         <is>
-          <t>Оплачено 80,450 USD (6 поз.). Даже небольшой платёж греет, как лавандовый раф в холодный день 🌸</t>
+          <t>Пришло 80 450 USD. Не фейерверк — зато честный сладкий момент. Самый заметный платёж: 27 000 USD. Спасибо клиенту ✨</t>
         </is>
       </c>
       <c r="P61" s="28" t="n"/>
       <c r="Q61" s="28" t="n"/>
       <c r="R61" s="28" t="n"/>
     </row>
-    <row r="62" ht="18" customHeight="1">
+    <row r="62" ht="20" customHeight="1">
       <c r="A62" s="16" t="inlineStr">
         <is>
           <t>№ счета</t>
@@ -4424,7 +4432,7 @@
       <c r="Q62" s="28" t="n"/>
       <c r="R62" s="28" t="n"/>
     </row>
-    <row r="63" ht="18" customHeight="1">
+    <row r="63" ht="20" customHeight="1">
       <c r="A63" s="29" t="inlineStr">
         <is>
           <t>8062610160-4</t>
@@ -4471,7 +4479,7 @@
       <c r="Q63" s="28" t="n"/>
       <c r="R63" s="28" t="n"/>
     </row>
-    <row r="64" ht="18" customHeight="1">
+    <row r="64" ht="20" customHeight="1">
       <c r="A64" s="29" t="n">
         <v>22062615414</v>
       </c>
@@ -4516,7 +4524,7 @@
       <c r="Q64" s="28" t="n"/>
       <c r="R64" s="28" t="n"/>
     </row>
-    <row r="65">
+    <row r="65" ht="20" customHeight="1">
       <c r="A65" s="29" t="inlineStr">
         <is>
           <t>18062615004</t>
@@ -4558,6 +4566,10 @@
           <t>этап 2 в периоде</t>
         </is>
       </c>
+      <c r="O65" s="28" t="n"/>
+      <c r="P65" s="28" t="n"/>
+      <c r="Q65" s="28" t="n"/>
+      <c r="R65" s="28" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="29" t="n">
@@ -4694,19 +4706,19 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A60:M60"/>
-    <mergeCell ref="O61:R64"/>
+    <mergeCell ref="O61:R65"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="O4:R4"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="O21:R25"/>
     <mergeCell ref="O60:R60"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="O21:R24"/>
+    <mergeCell ref="O5:R9"/>
     <mergeCell ref="O20:R20"/>
-    <mergeCell ref="A61:H61"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A20:M20"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="O5:R8"/>
+    <mergeCell ref="A61:H61"/>
     <mergeCell ref="A71:M71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>